<commit_message>
Hinos Antigos: opção hinário + pendrive com as músicas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Syb2BntMxVm3BZmSsihore
</commit_message>
<xml_diff>
--- a/catalogo-revisao.xlsx
+++ b/catalogo-revisao.xlsx
@@ -1814,7 +1814,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Músicas gravadas</t>
+          <t>Hinário + pendrive com as músicas</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr"/>
       <c r="G35" s="6" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>

</xml_diff>